<commit_message>
Fix the comparison of input files with git files
Also, add 6-benzyladenine aquatic toxicity as recorded by Marcel and add
the input files that were not included/updated because of the bugs
in the git comparison routines.
</commit_message>
<xml_diff>
--- a/data_generation/10_aquatic_toxicity/tebuconazole_aquatic_toxicity.xlsx
+++ b/data_generation/10_aquatic_toxicity/tebuconazole_aquatic_toxicity.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\10_aquatic_toxicity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F523204-896F-46BA-BE29-D459F45A5F6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96D5C3D3-4AAF-4034-9B33-756C36C174D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-13068" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="aquatic_endpoints" sheetId="6" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="88">
   <si>
     <t>Oncorhynchus mykiss</t>
   </si>
@@ -183,9 +183,6 @@
     <t>21 d</t>
   </si>
   <si>
-    <t>j.efsa.2009.296r</t>
-  </si>
-  <si>
     <t>rajo</t>
   </si>
   <si>
@@ -298,6 +295,12 @@
   </si>
   <si>
     <t>other</t>
+  </si>
+  <si>
+    <t>j.efsa.2014.3485</t>
+  </si>
+  <si>
+    <t>mamr</t>
   </si>
 </sst>
 </file>
@@ -327,12 +330,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -347,7 +356,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -373,6 +382,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -656,28 +668,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C316ADCA-0F97-4E34-A600-B1604EAF90B0}">
   <dimension ref="A1:X43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.42578125" defaultRowHeight="15.6" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.453125" defaultRowHeight="15.65" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" style="4" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" style="4" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="7.42578125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="14.7265625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="19.7265625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="7.453125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" style="4" customWidth="1"/>
     <col min="6" max="6" width="12" style="4" customWidth="1"/>
-    <col min="7" max="8" width="9.42578125" style="4"/>
-    <col min="9" max="9" width="9.42578125" style="4" customWidth="1"/>
-    <col min="10" max="11" width="9.42578125" style="4"/>
-    <col min="12" max="12" width="5.5703125" style="4" customWidth="1"/>
-    <col min="13" max="15" width="9.42578125" style="4"/>
-    <col min="16" max="16" width="17.42578125" style="4" customWidth="1"/>
-    <col min="17" max="17" width="9.42578125" style="4"/>
-    <col min="18" max="18" width="14.28515625" style="4" customWidth="1"/>
-    <col min="19" max="19" width="13.140625" style="4" customWidth="1"/>
-    <col min="20" max="20" width="9.42578125" style="5"/>
-    <col min="21" max="16384" width="9.42578125" style="4"/>
+    <col min="7" max="8" width="9.453125" style="4"/>
+    <col min="9" max="9" width="9.453125" style="4" customWidth="1"/>
+    <col min="10" max="11" width="9.453125" style="4"/>
+    <col min="12" max="12" width="5.54296875" style="4" customWidth="1"/>
+    <col min="13" max="15" width="9.453125" style="4"/>
+    <col min="16" max="16" width="17.453125" style="4" customWidth="1"/>
+    <col min="17" max="17" width="9.453125" style="4"/>
+    <col min="18" max="18" width="14.26953125" style="4" customWidth="1"/>
+    <col min="19" max="19" width="13.1796875" style="4" customWidth="1"/>
+    <col min="20" max="20" width="9.453125" style="5"/>
+    <col min="21" max="16384" width="9.453125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" s="1" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>23</v>
       </c>
@@ -730,10 +742,10 @@
         <v>15</v>
       </c>
       <c r="R1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="S1" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="T1" s="2" t="s">
         <v>17</v>
@@ -751,12 +763,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>54</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>0</v>
@@ -780,7 +792,7 @@
         <v>1</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M2" s="11">
         <v>4.4000000000000004</v>
@@ -791,14 +803,14 @@
       <c r="O2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="P2" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q2" s="3">
-        <v>83</v>
+      <c r="P2" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q2" s="13">
+        <v>73</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S2" s="3">
         <v>56</v>
@@ -811,16 +823,18 @@
       </c>
       <c r="V2" s="3"/>
       <c r="W2" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X2" s="3"/>
-    </row>
-    <row r="3" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>54</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>0</v>
@@ -844,7 +858,7 @@
         <v>1</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M3" s="12">
         <v>2.2999999999999998</v>
@@ -855,14 +869,14 @@
       <c r="O3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="P3" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q3" s="3">
-        <v>83</v>
+      <c r="P3" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q3" s="13">
+        <v>73</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S3" s="3">
         <v>57</v>
@@ -875,16 +889,18 @@
       </c>
       <c r="V3" s="3"/>
       <c r="W3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X3" s="3"/>
-    </row>
-    <row r="4" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X3" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>54</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>2</v>
@@ -902,7 +918,7 @@
         <v>3</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M4" s="9">
         <v>1.9</v>
@@ -913,14 +929,14 @@
       <c r="O4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="P4" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q4" s="3">
-        <v>83</v>
+      <c r="P4" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q4" s="13">
+        <v>73</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S4" s="3">
         <v>73</v>
@@ -932,19 +948,21 @@
         <v>44</v>
       </c>
       <c r="W4" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X4" s="6"/>
-    </row>
-    <row r="5" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X4" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>54</v>
-      </c>
       <c r="C5" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D5" s="3">
         <v>4</v>
@@ -962,7 +980,7 @@
         <v>3</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M5" s="9">
         <v>3.45</v>
@@ -973,14 +991,14 @@
       <c r="O5" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="P5" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q5" s="3">
-        <v>83</v>
+      <c r="P5" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q5" s="13">
+        <v>73</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S5" s="3">
         <v>85</v>
@@ -992,19 +1010,21 @@
         <v>44</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X5" s="6"/>
-    </row>
-    <row r="6" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X5" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>54</v>
-      </c>
       <c r="C6" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D6" s="3">
         <v>4</v>
@@ -1022,7 +1042,7 @@
         <v>3</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M6" s="9">
         <v>5.83</v>
@@ -1033,14 +1053,14 @@
       <c r="O6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="P6" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q6" s="3">
-        <v>83</v>
+      <c r="P6" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q6" s="13">
+        <v>73</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S6" s="3">
         <v>85</v>
@@ -1052,13 +1072,15 @@
         <v>44</v>
       </c>
       <c r="W6" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X6" s="6"/>
-    </row>
-    <row r="7" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X6" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>0</v>
@@ -1079,7 +1101,7 @@
         <v>1</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M7" s="10">
         <v>4.4000000000000004</v>
@@ -1090,14 +1112,14 @@
       <c r="O7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="P7" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q7" s="3">
-        <v>83</v>
+      <c r="P7" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q7" s="13">
+        <v>73</v>
       </c>
       <c r="R7" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S7" s="3">
         <v>53</v>
@@ -1110,16 +1132,18 @@
       </c>
       <c r="V7" s="3"/>
       <c r="W7" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X7" s="6"/>
-    </row>
-    <row r="8" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X7" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D8" s="3">
         <v>6</v>
@@ -1137,7 +1161,7 @@
         <v>1</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M8" s="10">
         <v>5.7</v>
@@ -1148,14 +1172,14 @@
       <c r="O8" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="P8" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q8" s="3">
-        <v>83</v>
+      <c r="P8" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q8" s="13">
+        <v>73</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S8" s="3">
         <v>54</v>
@@ -1168,16 +1192,18 @@
       </c>
       <c r="V8" s="3"/>
       <c r="W8" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X8" s="6"/>
-    </row>
-    <row r="9" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X8" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D9" s="3">
         <v>7</v>
@@ -1195,7 +1221,7 @@
         <v>1</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M9" s="10">
         <v>8.6999999999999993</v>
@@ -1206,14 +1232,14 @@
       <c r="O9" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="P9" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q9" s="3">
-        <v>83</v>
+      <c r="P9" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q9" s="13">
+        <v>73</v>
       </c>
       <c r="R9" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S9" s="3">
         <v>51</v>
@@ -1226,13 +1252,15 @@
       </c>
       <c r="V9" s="3"/>
       <c r="W9" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X9" s="6"/>
-    </row>
-    <row r="10" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X9" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>0</v>
@@ -1250,7 +1278,7 @@
         <v>42</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M10" s="10">
         <v>0.01</v>
@@ -1261,14 +1289,14 @@
       <c r="O10" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="P10" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q10" s="3">
-        <v>83</v>
+      <c r="P10" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q10" s="13">
+        <v>73</v>
       </c>
       <c r="R10" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S10" s="3">
         <v>61</v>
@@ -1281,13 +1309,15 @@
       </c>
       <c r="V10" s="3"/>
       <c r="W10" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X10" s="6"/>
-    </row>
-    <row r="11" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X10" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>0</v>
@@ -1299,7 +1329,7 @@
         <v>38</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>40</v>
@@ -1308,7 +1338,7 @@
         <v>42</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M11" s="10">
         <v>1.2E-2</v>
@@ -1319,14 +1349,14 @@
       <c r="O11" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="P11" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q11" s="3">
-        <v>83</v>
+      <c r="P11" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q11" s="13">
+        <v>73</v>
       </c>
       <c r="R11" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S11" s="6">
         <v>65</v>
@@ -1338,16 +1368,18 @@
         <v>44</v>
       </c>
       <c r="W11" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X11" s="6"/>
-    </row>
-    <row r="12" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X11" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D12" s="6">
         <v>10</v>
@@ -1356,13 +1388,13 @@
         <v>38</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K12" s="4" t="s">
         <v>42</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M12" s="10">
         <v>6.2500000000000003E-3</v>
@@ -1370,11 +1402,11 @@
       <c r="N12" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="P12" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q12" s="3">
-        <v>83</v>
+      <c r="P12" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q12" s="13">
+        <v>73</v>
       </c>
       <c r="R12" s="6"/>
       <c r="S12" s="6"/>
@@ -1385,16 +1417,18 @@
         <v>44</v>
       </c>
       <c r="W12" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X12" s="6"/>
-    </row>
-    <row r="13" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X12" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D13" s="6">
         <v>10</v>
@@ -1403,13 +1437,13 @@
         <v>38</v>
       </c>
       <c r="G13" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="K13" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="K13" s="4" t="s">
-        <v>63</v>
-      </c>
       <c r="L13" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M13" s="10">
         <v>1.2500000000000001E-2</v>
@@ -1417,31 +1451,33 @@
       <c r="N13" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="P13" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q13" s="3">
-        <v>83</v>
+      <c r="P13" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q13" s="13">
+        <v>73</v>
       </c>
       <c r="R13" s="6"/>
       <c r="S13" s="6"/>
       <c r="T13" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="U13" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="W13" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="X13" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>64</v>
-      </c>
-      <c r="W13" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X13" s="6"/>
-    </row>
-    <row r="14" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>65</v>
       </c>
       <c r="D14" s="6">
         <v>11</v>
@@ -1450,22 +1486,22 @@
         <v>38</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>40</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>42</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M14" s="10">
         <v>2.1899999999999999E-2</v>
@@ -1476,14 +1512,14 @@
       <c r="O14" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="P14" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q14" s="3">
-        <v>83</v>
+      <c r="P14" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q14" s="13">
+        <v>73</v>
       </c>
       <c r="R14" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S14" s="6">
         <v>66</v>
@@ -1495,16 +1531,18 @@
         <v>44</v>
       </c>
       <c r="W14" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X14" s="6"/>
-    </row>
-    <row r="15" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X14" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D15" s="6">
         <v>12</v>
@@ -1513,19 +1551,19 @@
         <v>38</v>
       </c>
       <c r="G15" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="I15" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>70</v>
       </c>
       <c r="K15" s="4" t="s">
         <v>42</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M15" s="10">
         <v>4.36E-2</v>
@@ -1536,14 +1574,14 @@
       <c r="O15" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="P15" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q15" s="3">
-        <v>83</v>
+      <c r="P15" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q15" s="13">
+        <v>73</v>
       </c>
       <c r="R15" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S15" s="6">
         <v>68</v>
@@ -1555,13 +1593,15 @@
         <v>44</v>
       </c>
       <c r="W15" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X15" s="6"/>
-    </row>
-    <row r="16" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X15" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>2</v>
@@ -1579,7 +1619,7 @@
         <v>3</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M16" s="10">
         <v>2.79</v>
@@ -1590,14 +1630,14 @@
       <c r="O16" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="P16" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q16" s="3">
-        <v>84</v>
+      <c r="P16" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q16" s="13">
+        <v>74</v>
       </c>
       <c r="R16" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S16" s="6">
         <v>71</v>
@@ -1609,13 +1649,15 @@
         <v>44</v>
       </c>
       <c r="W16" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X16" s="6"/>
-    </row>
-    <row r="17" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X16" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>2</v>
@@ -1633,7 +1675,7 @@
         <v>42</v>
       </c>
       <c r="L17" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M17" s="10">
         <v>0.12</v>
@@ -1644,14 +1686,14 @@
       <c r="O17" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="P17" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q17" s="3">
-        <v>84</v>
+      <c r="P17" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q17" s="13">
+        <v>74</v>
       </c>
       <c r="R17" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S17" s="6">
         <v>78</v>
@@ -1663,13 +1705,15 @@
         <v>44</v>
       </c>
       <c r="W17" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X17" s="6"/>
-    </row>
-    <row r="18" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X17" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>2</v>
@@ -1687,7 +1731,7 @@
         <v>42</v>
       </c>
       <c r="L18" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M18" s="10">
         <v>0.1</v>
@@ -1698,14 +1742,14 @@
       <c r="O18" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="P18" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q18" s="3">
-        <v>84</v>
+      <c r="P18" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q18" s="13">
+        <v>74</v>
       </c>
       <c r="R18" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S18" s="6">
         <v>80</v>
@@ -1714,16 +1758,18 @@
         <v>10</v>
       </c>
       <c r="U18" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W18" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X18" s="6"/>
-    </row>
-    <row r="19" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X18" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>2</v>
@@ -1732,10 +1778,10 @@
         <v>16</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K19" s="4" t="s">
         <v>42</v>
@@ -1749,30 +1795,32 @@
       <c r="N19" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="P19" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q19" s="3">
-        <v>84</v>
+      <c r="P19" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q19" s="13">
+        <v>74</v>
       </c>
       <c r="R19" s="3"/>
       <c r="T19" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="U19" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="W19" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X19" s="6"/>
-    </row>
-    <row r="20" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X19" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D20" s="6">
         <v>17</v>
@@ -1781,19 +1829,19 @@
         <v>5</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>37</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K20" s="4" t="s">
         <v>42</v>
       </c>
       <c r="L20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="M20" s="10">
         <v>0.1</v>
@@ -1804,14 +1852,14 @@
       <c r="O20" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="P20" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q20" s="3">
-        <v>84</v>
+      <c r="P20" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q20" s="13">
+        <v>74</v>
       </c>
       <c r="R20" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S20" s="6">
         <v>90</v>
@@ -1823,19 +1871,21 @@
         <v>44</v>
       </c>
       <c r="V20" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="W20" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X20" s="6"/>
-    </row>
-    <row r="21" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X20" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D21" s="6">
         <v>18</v>
@@ -1844,19 +1894,19 @@
         <v>5</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>37</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M21" s="10">
         <v>2.4500000000000002</v>
@@ -1867,14 +1917,14 @@
       <c r="O21" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="P21" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q21" s="3">
-        <v>84</v>
+      <c r="P21" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q21" s="13">
+        <v>74</v>
       </c>
       <c r="R21" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S21" s="6">
         <v>91</v>
@@ -1886,16 +1936,18 @@
         <v>44</v>
       </c>
       <c r="W21" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X21" s="6"/>
-    </row>
-    <row r="22" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X21" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D22" s="6">
         <v>19</v>
@@ -1904,34 +1956,36 @@
         <v>5</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="M22" s="9"/>
-      <c r="P22" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q22" s="3">
-        <v>84</v>
+      <c r="P22" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q22" s="13">
+        <v>74</v>
       </c>
       <c r="R22" s="3"/>
       <c r="S22" s="6"/>
       <c r="T22" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="U22" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="W22" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X22" s="6"/>
-    </row>
-    <row r="23" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X22" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D23" s="6">
         <v>20</v>
@@ -1949,7 +2003,7 @@
         <v>3</v>
       </c>
       <c r="L23" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M23" s="9">
         <v>1.96</v>
@@ -1960,14 +2014,14 @@
       <c r="O23" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="P23" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q23" s="3">
-        <v>84</v>
+      <c r="P23" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q23" s="13">
+        <v>74</v>
       </c>
       <c r="R23" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S23" s="6">
         <v>83</v>
@@ -1979,16 +2033,18 @@
         <v>44</v>
       </c>
       <c r="W23" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X23" s="6"/>
-    </row>
-    <row r="24" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X23" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D24" s="6">
         <v>20</v>
@@ -2006,7 +2062,7 @@
         <v>3</v>
       </c>
       <c r="L24" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M24" s="9">
         <v>5.3</v>
@@ -2017,14 +2073,14 @@
       <c r="O24" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="P24" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q24" s="3">
-        <v>84</v>
+      <c r="P24" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q24" s="13">
+        <v>74</v>
       </c>
       <c r="R24" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S24" s="6">
         <v>83</v>
@@ -2036,13 +2092,15 @@
         <v>44</v>
       </c>
       <c r="W24" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X24" s="6"/>
-    </row>
-    <row r="25" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X24" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>46</v>
@@ -2063,7 +2121,7 @@
         <v>3</v>
       </c>
       <c r="L25" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M25" s="9">
         <v>2.83</v>
@@ -2074,14 +2132,14 @@
       <c r="O25" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="P25" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q25" s="3">
-        <v>84</v>
+      <c r="P25" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q25" s="13">
+        <v>74</v>
       </c>
       <c r="R25" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S25" s="6">
         <v>84</v>
@@ -2093,13 +2151,15 @@
         <v>44</v>
       </c>
       <c r="W25" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X25" s="6"/>
-    </row>
-    <row r="26" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X25" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="26" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>46</v>
@@ -2120,7 +2180,7 @@
         <v>3</v>
       </c>
       <c r="L26" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M26" s="9">
         <v>3.8</v>
@@ -2131,14 +2191,14 @@
       <c r="O26" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="P26" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q26" s="3">
-        <v>84</v>
+      <c r="P26" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q26" s="13">
+        <v>74</v>
       </c>
       <c r="R26" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S26" s="6">
         <v>84</v>
@@ -2150,16 +2210,18 @@
         <v>44</v>
       </c>
       <c r="W26" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X26" s="6"/>
-    </row>
-    <row r="27" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X26" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D27" s="6">
         <v>22</v>
@@ -2171,16 +2233,16 @@
         <v>20</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K27" s="4" t="s">
         <v>3</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M27" s="9">
         <v>3</v>
@@ -2191,14 +2253,14 @@
       <c r="O27" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="P27" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q27" s="3">
-        <v>84</v>
+      <c r="P27" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q27" s="13">
+        <v>74</v>
       </c>
       <c r="R27" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S27" s="6">
         <v>77</v>
@@ -2210,16 +2272,18 @@
         <v>44</v>
       </c>
       <c r="W27" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X27" s="6"/>
-    </row>
-    <row r="28" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X27" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D28" s="6">
         <v>23</v>
@@ -2238,7 +2302,7 @@
         <v>1</v>
       </c>
       <c r="L28" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M28" s="10">
         <v>0.46</v>
@@ -2249,14 +2313,14 @@
       <c r="O28" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="P28" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q28" s="3">
-        <v>84</v>
+      <c r="P28" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q28" s="13">
+        <v>74</v>
       </c>
       <c r="R28" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S28" s="6">
         <v>78</v>
@@ -2268,16 +2332,18 @@
         <v>44</v>
       </c>
       <c r="W28" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X28" s="6"/>
-    </row>
-    <row r="29" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X28" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D29" s="6">
         <v>24</v>
@@ -2295,7 +2361,7 @@
         <v>42</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M29" s="10">
         <v>3.5000000000000003E-2</v>
@@ -2306,14 +2372,14 @@
       <c r="O29" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="P29" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q29" s="3">
-        <v>84</v>
+      <c r="P29" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q29" s="13">
+        <v>74</v>
       </c>
       <c r="R29" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S29" s="6">
         <v>82</v>
@@ -2325,11 +2391,13 @@
         <v>44</v>
       </c>
       <c r="W29" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X29" s="6"/>
-    </row>
-    <row r="30" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="X29" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="30" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D30" s="6"/>
       <c r="M30" s="9"/>
       <c r="Q30" s="6"/>
@@ -2340,7 +2408,7 @@
       <c r="W30" s="3"/>
       <c r="X30" s="6"/>
     </row>
-    <row r="31" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D31" s="6"/>
       <c r="M31" s="9"/>
       <c r="Q31" s="6"/>
@@ -2351,40 +2419,40 @@
       <c r="W31" s="3"/>
       <c r="X31" s="6"/>
     </row>
-    <row r="32" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:24" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M32" s="9"/>
     </row>
-    <row r="33" spans="13:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="13:13" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M33" s="9"/>
     </row>
-    <row r="34" spans="13:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="13:13" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M34" s="9"/>
     </row>
-    <row r="35" spans="13:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="13:13" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M35" s="9"/>
     </row>
-    <row r="36" spans="13:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="13:13" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M36" s="9"/>
     </row>
-    <row r="37" spans="13:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="13:13" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M37" s="9"/>
     </row>
-    <row r="38" spans="13:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="13:13" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M38" s="9"/>
     </row>
-    <row r="39" spans="13:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="13:13" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M39" s="9"/>
     </row>
-    <row r="40" spans="13:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="13:13" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M40" s="9"/>
     </row>
-    <row r="41" spans="13:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="13:13" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M41" s="9"/>
     </row>
-    <row r="42" spans="13:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="13:13" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M42" s="9"/>
     </row>
-    <row r="43" spans="13:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="13:13" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M43" s="9"/>
     </row>
   </sheetData>

</xml_diff>